<commit_message>
feb 16 add ,imtes to click changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeClockRecorderForFVAStandardUserOnSFLightningView.xlsx
+++ b/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeClockRecorderForFVAStandardUserOnSFLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F69CB5DA-2CD4-4BDB-86A5-937C74F3D27E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAC747F-AFA4-440A-B4C6-55AA921E7F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="ModuleName" sheetId="13" r:id="rId3"/>
     <sheet name="TimeClockRecorder" sheetId="7" r:id="rId4"/>
     <sheet name="UpdateData" sheetId="14" r:id="rId5"/>
-    <sheet name="TimeClockRecorder2" sheetId="15" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Global Search User</t>
   </si>
@@ -113,6 +112,12 @@
   </si>
   <si>
     <t>LogTIme</t>
+  </si>
+  <si>
+    <t>Additional Minutes</t>
+  </si>
+  <si>
+    <t>120</t>
   </si>
 </sst>
 </file>
@@ -549,7 +554,7 @@
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="43.28515625" customWidth="1"/>
   </cols>
@@ -567,7 +572,9 @@
       <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -583,7 +590,9 @@
       <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3"/>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -598,6 +607,9 @@
       </c>
       <c r="D3" s="4" t="s">
         <v>19</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -643,32 +655,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA8B519D-B6C7-4E9E-B893-5442930BCAA2}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
TMTT0005211- Feb 28 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeClockRecorderForFVAStandardUserOnSFLightningView.xlsx
+++ b/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeClockRecorderForFVAStandardUserOnSFLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAC747F-AFA4-440A-B4C6-55AA921E7F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA1E31A-A7B5-45BC-823F-D7274E9302E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -72,12 +72,6 @@
     <t>Time Record Manager</t>
   </si>
   <si>
-    <t>Cindy Ma</t>
-  </si>
-  <si>
-    <t>Abax Credit Fund III-Abax Global Capital-FVA-104456</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -90,9 +84,6 @@
     <t>GroupName</t>
   </si>
   <si>
-    <t>Time Tracking PV</t>
-  </si>
-  <si>
     <t>Profile</t>
   </si>
   <si>
@@ -102,15 +93,6 @@
     <t>Time Record Period:</t>
   </si>
   <si>
-    <t>Rachel Du</t>
-  </si>
-  <si>
-    <t>Time Tracking PV Supervisor</t>
-  </si>
-  <si>
-    <t>Abax FY2014-Abax Global Capital-FVA-22406</t>
-  </si>
-  <si>
     <t>LogTIme</t>
   </si>
   <si>
@@ -118,6 +100,24 @@
   </si>
   <si>
     <t>120</t>
+  </si>
+  <si>
+    <t>Amy Xia</t>
+  </si>
+  <si>
+    <t>Time Tracking Litigation</t>
+  </si>
+  <si>
+    <t>Debevoise_Xie (Compo Expert)-Debevoise &amp; Plimpton LLP-FVA-26522</t>
+  </si>
+  <si>
+    <t>Ashley Choi</t>
+  </si>
+  <si>
+    <t>MEH) Thompson_CLP Toxicology-Thompson Hine, LLP-FVA-26495</t>
+  </si>
+  <si>
+    <t>Time Tracking Litigation Supervisor</t>
   </si>
 </sst>
 </file>
@@ -156,7 +156,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -164,11 +164,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -176,6 +191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,7 +476,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -469,32 +485,32 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -551,8 +567,8 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
     <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -564,7 +580,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -573,43 +589,43 @@
         <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
+      <c r="A2" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -638,18 +654,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>